<commit_message>
Reverify D5 instrument inventory evidence
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D5 Topological Role Consistency and Structural Representativeness/outputs/local/D5_case_study_exports.xlsx
+++ b/Project 1 Data Quality Assessment/D5 Topological Role Consistency and Structural Representativeness/outputs/local/D5_case_study_exports.xlsx
@@ -811,7 +811,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q2" t="n">
@@ -921,7 +921,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q3" t="n">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q4" t="n">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q5" t="n">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q6" t="n">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1371,7 +1371,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q7" t="n">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q8" t="n">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q9" t="n">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1701,7 +1701,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q10" t="n">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q11" t="n">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q12" t="n">
@@ -2021,7 +2021,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q13" t="n">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q14" t="n">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q15" t="n">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -2361,7 +2361,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q16" t="n">
@@ -2461,7 +2461,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q17" t="n">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q18" t="n">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q19" t="n">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q20" t="n">
@@ -2901,7 +2901,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q21" t="n">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q22" t="n">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q23" t="n">
@@ -3231,7 +3231,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q24" t="n">
@@ -3341,7 +3341,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -3351,7 +3351,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q25" t="n">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -3461,7 +3461,7 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q26" t="n">
@@ -3561,7 +3561,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q27" t="n">
@@ -3671,7 +3671,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -3681,7 +3681,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q28" t="n">
@@ -3781,7 +3781,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -3791,7 +3791,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q29" t="n">
@@ -3891,7 +3891,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q30" t="n">
@@ -4001,7 +4001,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -4011,7 +4011,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q31" t="n">
@@ -4111,7 +4111,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -4121,7 +4121,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q32" t="n">
@@ -4221,7 +4221,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -4231,7 +4231,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q33" t="n">
@@ -4331,7 +4331,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q34" t="n">
@@ -4441,7 +4441,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
@@ -4451,7 +4451,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q35" t="n">
@@ -4551,7 +4551,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
@@ -4561,7 +4561,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q36" t="n">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q37" t="n">
@@ -4771,7 +4771,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
@@ -4781,7 +4781,7 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q38" t="n">
@@ -4881,7 +4881,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -4891,7 +4891,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q39" t="n">
@@ -4991,7 +4991,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q40" t="n">
@@ -5101,7 +5101,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
@@ -5111,7 +5111,7 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q41" t="n">
@@ -5211,7 +5211,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
@@ -5221,7 +5221,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q42" t="n">
@@ -5321,7 +5321,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q43" t="n">
@@ -5431,7 +5431,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
@@ -5441,7 +5441,7 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q44" t="n">
@@ -5541,7 +5541,7 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
@@ -5551,7 +5551,7 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q45" t="n">
@@ -5651,7 +5651,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
@@ -5661,7 +5661,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q46" t="n">
@@ -5761,7 +5761,7 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
@@ -5771,7 +5771,7 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q47" t="n">
@@ -5871,7 +5871,7 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
@@ -5881,7 +5881,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q48" t="n">
@@ -5981,7 +5981,7 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
@@ -5991,7 +5991,7 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q49" t="n">
@@ -6091,7 +6091,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
@@ -6101,7 +6101,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q50" t="n">
@@ -6201,7 +6201,7 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q51" t="n">
@@ -6311,7 +6311,7 @@
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
@@ -6321,7 +6321,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q52" t="n">
@@ -6421,7 +6421,7 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
@@ -6431,7 +6431,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q53" t="n">
@@ -6531,7 +6531,7 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
@@ -6541,7 +6541,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q54" t="n">
@@ -6641,7 +6641,7 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
@@ -6651,7 +6651,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q55" t="n">
@@ -6751,7 +6751,7 @@
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
@@ -6761,7 +6761,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q56" t="n">
@@ -6861,7 +6861,7 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
@@ -6871,7 +6871,7 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q57" t="n">
@@ -6971,7 +6971,7 @@
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
@@ -6981,7 +6981,7 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q58" t="n">
@@ -7081,7 +7081,7 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
@@ -7091,7 +7091,7 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q59" t="n">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
@@ -7201,7 +7201,7 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q60" t="n">
@@ -7301,7 +7301,7 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
@@ -7311,7 +7311,7 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q61" t="n">
@@ -7411,7 +7411,7 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
@@ -7421,7 +7421,7 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q62" t="n">
@@ -7521,7 +7521,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
@@ -7531,7 +7531,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q63" t="n">
@@ -7631,7 +7631,7 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O64" t="inlineStr">
@@ -7641,7 +7641,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q64" t="n">
@@ -7741,7 +7741,7 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O65" t="inlineStr">
@@ -7751,7 +7751,7 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q65" t="n">
@@ -7851,7 +7851,7 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O66" t="inlineStr">
@@ -7861,7 +7861,7 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q66" t="n">
@@ -7961,7 +7961,7 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
@@ -7971,7 +7971,7 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q67" t="n">
@@ -8071,7 +8071,7 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
@@ -8081,7 +8081,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q68" t="n">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
@@ -8191,7 +8191,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q69" t="n">
@@ -8291,7 +8291,7 @@
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
@@ -8301,7 +8301,7 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q70" t="n">
@@ -8401,7 +8401,7 @@
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
@@ -8411,7 +8411,7 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q71" t="n">
@@ -8511,7 +8511,7 @@
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
@@ -8521,7 +8521,7 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q72" t="n">
@@ -8621,7 +8621,7 @@
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
@@ -8631,7 +8631,7 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q73" t="n">
@@ -8731,7 +8731,7 @@
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
@@ -8741,7 +8741,7 @@
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q74" t="n">
@@ -8841,7 +8841,7 @@
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O75" t="inlineStr">
@@ -8851,7 +8851,7 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q75" t="n">
@@ -8951,7 +8951,7 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O76" t="inlineStr">
@@ -8961,7 +8961,7 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q76" t="n">
@@ -9061,7 +9061,7 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
@@ -9071,7 +9071,7 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q77" t="n">
@@ -9171,7 +9171,7 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
@@ -9181,7 +9181,7 @@
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q78" t="n">
@@ -9281,7 +9281,7 @@
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
@@ -9291,7 +9291,7 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q79" t="n">
@@ -9391,7 +9391,7 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
@@ -9401,7 +9401,7 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q80" t="n">
@@ -9501,7 +9501,7 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O81" t="inlineStr">
@@ -9511,7 +9511,7 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q81" t="n">
@@ -9611,7 +9611,7 @@
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O82" t="inlineStr">
@@ -9621,7 +9621,7 @@
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q82" t="n">
@@ -9721,7 +9721,7 @@
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O83" t="inlineStr">
@@ -9731,7 +9731,7 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q83" t="n">
@@ -9831,7 +9831,7 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O84" t="inlineStr">
@@ -9841,7 +9841,7 @@
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q84" t="n">
@@ -9941,7 +9941,7 @@
       </c>
       <c r="N85" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O85" t="inlineStr">
@@ -9951,7 +9951,7 @@
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q85" t="n">
@@ -10051,7 +10051,7 @@
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O86" t="inlineStr">
@@ -10061,7 +10061,7 @@
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q86" t="n">
@@ -10161,7 +10161,7 @@
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O87" t="inlineStr">
@@ -10171,7 +10171,7 @@
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q87" t="n">
@@ -10271,7 +10271,7 @@
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O88" t="inlineStr">
@@ -10281,7 +10281,7 @@
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q88" t="n">
@@ -10381,7 +10381,7 @@
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O89" t="inlineStr">
@@ -10391,7 +10391,7 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q89" t="n">
@@ -10491,7 +10491,7 @@
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O90" t="inlineStr">
@@ -10501,7 +10501,7 @@
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q90" t="n">
@@ -10601,7 +10601,7 @@
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O91" t="inlineStr">
@@ -10611,7 +10611,7 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q91" t="n">
@@ -10711,7 +10711,7 @@
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O92" t="inlineStr">
@@ -10721,7 +10721,7 @@
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q92" t="n">
@@ -10821,7 +10821,7 @@
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O93" t="inlineStr">
@@ -10831,7 +10831,7 @@
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q93" t="n">
@@ -10931,7 +10931,7 @@
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O94" t="inlineStr">
@@ -10941,7 +10941,7 @@
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q94" t="n">
@@ -11041,7 +11041,7 @@
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O95" t="inlineStr">
@@ -11051,7 +11051,7 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q95" t="n">
@@ -11151,7 +11151,7 @@
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O96" t="inlineStr">
@@ -11161,7 +11161,7 @@
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q96" t="n">
@@ -11261,7 +11261,7 @@
       </c>
       <c r="N97" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O97" t="inlineStr">
@@ -11271,7 +11271,7 @@
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q97" t="n">
@@ -11371,7 +11371,7 @@
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O98" t="inlineStr">
@@ -11381,7 +11381,7 @@
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q98" t="n">
@@ -11481,7 +11481,7 @@
       </c>
       <c r="N99" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O99" t="inlineStr">
@@ -11491,7 +11491,7 @@
       </c>
       <c r="P99" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q99" t="n">
@@ -11591,7 +11591,7 @@
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O100" t="inlineStr">
@@ -11601,7 +11601,7 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q100" t="n">
@@ -11701,7 +11701,7 @@
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O101" t="inlineStr">
@@ -11711,7 +11711,7 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q101" t="n">
@@ -11811,7 +11811,7 @@
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O102" t="inlineStr">
@@ -11821,7 +11821,7 @@
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q102" t="n">
@@ -11921,7 +11921,7 @@
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O103" t="inlineStr">
@@ -11931,7 +11931,7 @@
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q103" t="n">
@@ -12031,7 +12031,7 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O104" t="inlineStr">
@@ -12041,7 +12041,7 @@
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q104" t="n">
@@ -12141,7 +12141,7 @@
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O105" t="inlineStr">
@@ -12151,7 +12151,7 @@
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q105" t="n">
@@ -12251,7 +12251,7 @@
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O106" t="inlineStr">
@@ -12261,7 +12261,7 @@
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q106" t="n">
@@ -12361,7 +12361,7 @@
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O107" t="inlineStr">
@@ -12371,7 +12371,7 @@
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q107" t="n">
@@ -12471,7 +12471,7 @@
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O108" t="inlineStr">
@@ -12481,7 +12481,7 @@
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q108" t="n">
@@ -12581,7 +12581,7 @@
       </c>
       <c r="N109" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O109" t="inlineStr">
@@ -12591,7 +12591,7 @@
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q109" t="n">
@@ -12691,7 +12691,7 @@
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O110" t="inlineStr">
@@ -12701,7 +12701,7 @@
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q110" t="n">
@@ -12801,7 +12801,7 @@
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O111" t="inlineStr">
@@ -12811,7 +12811,7 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q111" t="n">
@@ -12911,7 +12911,7 @@
       </c>
       <c r="N112" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O112" t="inlineStr">
@@ -12921,7 +12921,7 @@
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q112" t="n">
@@ -13021,7 +13021,7 @@
       </c>
       <c r="N113" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O113" t="inlineStr">
@@ -13031,7 +13031,7 @@
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q113" t="n">
@@ -13131,7 +13131,7 @@
       </c>
       <c r="N114" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O114" t="inlineStr">
@@ -13141,7 +13141,7 @@
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q114" t="n">
@@ -13241,7 +13241,7 @@
       </c>
       <c r="N115" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O115" t="inlineStr">
@@ -13251,7 +13251,7 @@
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q115" t="n">
@@ -13351,7 +13351,7 @@
       </c>
       <c r="N116" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O116" t="inlineStr">
@@ -13361,7 +13361,7 @@
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q116" t="n">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="N117" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O117" t="inlineStr">
@@ -13471,7 +13471,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q117" t="n">
@@ -13571,7 +13571,7 @@
       </c>
       <c r="N118" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O118" t="inlineStr">
@@ -13581,7 +13581,7 @@
       </c>
       <c r="P118" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q118" t="n">
@@ -13681,7 +13681,7 @@
       </c>
       <c r="N119" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O119" t="inlineStr">
@@ -13691,7 +13691,7 @@
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q119" t="n">
@@ -13791,7 +13791,7 @@
       </c>
       <c r="N120" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O120" t="inlineStr">
@@ -13801,7 +13801,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q120" t="n">
@@ -13901,7 +13901,7 @@
       </c>
       <c r="N121" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O121" t="inlineStr">
@@ -13911,7 +13911,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q121" t="n">
@@ -14011,7 +14011,7 @@
       </c>
       <c r="N122" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O122" t="inlineStr">
@@ -14021,7 +14021,7 @@
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q122" t="n">
@@ -14121,7 +14121,7 @@
       </c>
       <c r="N123" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O123" t="inlineStr">
@@ -14131,7 +14131,7 @@
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q123" t="n">
@@ -14231,7 +14231,7 @@
       </c>
       <c r="N124" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O124" t="inlineStr">
@@ -14241,7 +14241,7 @@
       </c>
       <c r="P124" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q124" t="n">
@@ -14341,7 +14341,7 @@
       </c>
       <c r="N125" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O125" t="inlineStr">
@@ -14351,7 +14351,7 @@
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q125" t="n">
@@ -14451,7 +14451,7 @@
       </c>
       <c r="N126" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O126" t="inlineStr">
@@ -14461,7 +14461,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q126" t="n">
@@ -14561,7 +14561,7 @@
       </c>
       <c r="N127" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O127" t="inlineStr">
@@ -14571,7 +14571,7 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q127" t="n">
@@ -14671,7 +14671,7 @@
       </c>
       <c r="N128" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O128" t="inlineStr">
@@ -14681,7 +14681,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q128" t="n">
@@ -14781,7 +14781,7 @@
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O129" t="inlineStr">
@@ -14791,7 +14791,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q129" t="n">
@@ -14891,7 +14891,7 @@
       </c>
       <c r="N130" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O130" t="inlineStr">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q130" t="n">
@@ -15001,7 +15001,7 @@
       </c>
       <c r="N131" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O131" t="inlineStr">
@@ -15011,7 +15011,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q131" t="n">
@@ -15111,7 +15111,7 @@
       </c>
       <c r="N132" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O132" t="inlineStr">
@@ -15121,7 +15121,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q132" t="n">
@@ -15221,7 +15221,7 @@
       </c>
       <c r="N133" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O133" t="inlineStr">
@@ -15231,7 +15231,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q133" t="n">
@@ -15331,7 +15331,7 @@
       </c>
       <c r="N134" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O134" t="inlineStr">
@@ -15341,7 +15341,7 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q134" t="n">
@@ -15441,7 +15441,7 @@
       </c>
       <c r="N135" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O135" t="inlineStr">
@@ -15451,7 +15451,7 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q135" t="n">
@@ -15551,7 +15551,7 @@
       </c>
       <c r="N136" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O136" t="inlineStr">
@@ -15561,7 +15561,7 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q136" t="n">
@@ -15661,7 +15661,7 @@
       </c>
       <c r="N137" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O137" t="inlineStr">
@@ -15671,7 +15671,7 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q137" t="n">
@@ -15771,7 +15771,7 @@
       </c>
       <c r="N138" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O138" t="inlineStr">
@@ -15781,7 +15781,7 @@
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q138" t="n">
@@ -15881,7 +15881,7 @@
       </c>
       <c r="N139" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O139" t="inlineStr">
@@ -15891,7 +15891,7 @@
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q139" t="n">
@@ -15991,7 +15991,7 @@
       </c>
       <c r="N140" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O140" t="inlineStr">
@@ -16001,7 +16001,7 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q140" t="n">
@@ -16101,7 +16101,7 @@
       </c>
       <c r="N141" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O141" t="inlineStr">
@@ -16111,7 +16111,7 @@
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q141" t="n">
@@ -16211,7 +16211,7 @@
       </c>
       <c r="N142" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O142" t="inlineStr">
@@ -16221,7 +16221,7 @@
       </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q142" t="n">
@@ -16321,7 +16321,7 @@
       </c>
       <c r="N143" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O143" t="inlineStr">
@@ -16331,7 +16331,7 @@
       </c>
       <c r="P143" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q143" t="n">
@@ -16431,7 +16431,7 @@
       </c>
       <c r="N144" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O144" t="inlineStr">
@@ -16441,7 +16441,7 @@
       </c>
       <c r="P144" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q144" t="n">
@@ -16541,7 +16541,7 @@
       </c>
       <c r="N145" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O145" t="inlineStr">
@@ -16551,7 +16551,7 @@
       </c>
       <c r="P145" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q145" t="n">
@@ -16651,7 +16651,7 @@
       </c>
       <c r="N146" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O146" t="inlineStr">
@@ -16661,7 +16661,7 @@
       </c>
       <c r="P146" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q146" t="n">
@@ -16761,7 +16761,7 @@
       </c>
       <c r="N147" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O147" t="inlineStr">
@@ -16771,7 +16771,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q147" t="n">
@@ -16871,7 +16871,7 @@
       </c>
       <c r="N148" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O148" t="inlineStr">
@@ -16881,7 +16881,7 @@
       </c>
       <c r="P148" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q148" t="n">
@@ -16981,7 +16981,7 @@
       </c>
       <c r="N149" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O149" t="inlineStr">
@@ -16991,7 +16991,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q149" t="n">
@@ -17091,7 +17091,7 @@
       </c>
       <c r="N150" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O150" t="inlineStr">
@@ -17101,7 +17101,7 @@
       </c>
       <c r="P150" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q150" t="n">
@@ -17201,7 +17201,7 @@
       </c>
       <c r="N151" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O151" t="inlineStr">
@@ -17211,7 +17211,7 @@
       </c>
       <c r="P151" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q151" t="n">
@@ -17311,7 +17311,7 @@
       </c>
       <c r="N152" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O152" t="inlineStr">
@@ -17321,7 +17321,7 @@
       </c>
       <c r="P152" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q152" t="n">
@@ -17421,7 +17421,7 @@
       </c>
       <c r="N153" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O153" t="inlineStr">
@@ -17431,7 +17431,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q153" t="n">
@@ -17531,7 +17531,7 @@
       </c>
       <c r="N154" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O154" t="inlineStr">
@@ -17541,7 +17541,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q154" t="n">
@@ -17641,7 +17641,7 @@
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O155" t="inlineStr">
@@ -17651,7 +17651,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q155" t="n">
@@ -17751,7 +17751,7 @@
       </c>
       <c r="N156" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O156" t="inlineStr">
@@ -17761,7 +17761,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q156" t="n">
@@ -17861,7 +17861,7 @@
       </c>
       <c r="N157" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O157" t="inlineStr">
@@ -17871,7 +17871,7 @@
       </c>
       <c r="P157" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q157" t="n">
@@ -17971,7 +17971,7 @@
       </c>
       <c r="N158" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O158" t="inlineStr">
@@ -17981,7 +17981,7 @@
       </c>
       <c r="P158" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q158" t="n">
@@ -18081,7 +18081,7 @@
       </c>
       <c r="N159" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O159" t="inlineStr">
@@ -18091,7 +18091,7 @@
       </c>
       <c r="P159" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q159" t="n">
@@ -18191,7 +18191,7 @@
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O160" t="inlineStr">
@@ -18201,7 +18201,7 @@
       </c>
       <c r="P160" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q160" t="n">
@@ -18301,7 +18301,7 @@
       </c>
       <c r="N161" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O161" t="inlineStr">
@@ -18311,7 +18311,7 @@
       </c>
       <c r="P161" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q161" t="n">
@@ -18411,7 +18411,7 @@
       </c>
       <c r="N162" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O162" t="inlineStr">
@@ -18421,7 +18421,7 @@
       </c>
       <c r="P162" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q162" t="n">
@@ -18521,7 +18521,7 @@
       </c>
       <c r="N163" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O163" t="inlineStr">
@@ -18531,7 +18531,7 @@
       </c>
       <c r="P163" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q163" t="n">
@@ -18631,7 +18631,7 @@
       </c>
       <c r="N164" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O164" t="inlineStr">
@@ -18641,7 +18641,7 @@
       </c>
       <c r="P164" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q164" t="n">
@@ -18741,7 +18741,7 @@
       </c>
       <c r="N165" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O165" t="inlineStr">
@@ -18751,7 +18751,7 @@
       </c>
       <c r="P165" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q165" t="n">
@@ -18851,7 +18851,7 @@
       </c>
       <c r="N166" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O166" t="inlineStr">
@@ -18861,7 +18861,7 @@
       </c>
       <c r="P166" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q166" t="n">
@@ -18961,7 +18961,7 @@
       </c>
       <c r="N167" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O167" t="inlineStr">
@@ -18971,7 +18971,7 @@
       </c>
       <c r="P167" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q167" t="n">
@@ -19071,7 +19071,7 @@
       </c>
       <c r="N168" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O168" t="inlineStr">
@@ -19081,7 +19081,7 @@
       </c>
       <c r="P168" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q168" t="n">
@@ -19181,7 +19181,7 @@
       </c>
       <c r="N169" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O169" t="inlineStr">
@@ -19191,7 +19191,7 @@
       </c>
       <c r="P169" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q169" t="n">
@@ -19291,7 +19291,7 @@
       </c>
       <c r="N170" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O170" t="inlineStr">
@@ -19301,7 +19301,7 @@
       </c>
       <c r="P170" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q170" t="n">
@@ -19401,7 +19401,7 @@
       </c>
       <c r="N171" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O171" t="inlineStr">
@@ -19411,7 +19411,7 @@
       </c>
       <c r="P171" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q171" t="n">
@@ -19511,7 +19511,7 @@
       </c>
       <c r="N172" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O172" t="inlineStr">
@@ -19521,7 +19521,7 @@
       </c>
       <c r="P172" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q172" t="n">
@@ -19621,7 +19621,7 @@
       </c>
       <c r="N173" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O173" t="inlineStr">
@@ -19631,7 +19631,7 @@
       </c>
       <c r="P173" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q173" t="n">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="N174" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O174" t="inlineStr">
@@ -19741,7 +19741,7 @@
       </c>
       <c r="P174" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q174" t="n">
@@ -19841,7 +19841,7 @@
       </c>
       <c r="N175" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O175" t="inlineStr">
@@ -19851,7 +19851,7 @@
       </c>
       <c r="P175" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q175" t="n">
@@ -19951,7 +19951,7 @@
       </c>
       <c r="N176" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O176" t="inlineStr">
@@ -19961,7 +19961,7 @@
       </c>
       <c r="P176" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q176" t="n">
@@ -20061,7 +20061,7 @@
       </c>
       <c r="N177" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O177" t="inlineStr">
@@ -20071,7 +20071,7 @@
       </c>
       <c r="P177" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q177" t="n">
@@ -20171,7 +20171,7 @@
       </c>
       <c r="N178" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O178" t="inlineStr">
@@ -20181,7 +20181,7 @@
       </c>
       <c r="P178" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q178" t="n">
@@ -20281,7 +20281,7 @@
       </c>
       <c r="N179" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O179" t="inlineStr">
@@ -20291,7 +20291,7 @@
       </c>
       <c r="P179" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q179" t="n">
@@ -20391,7 +20391,7 @@
       </c>
       <c r="N180" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O180" t="inlineStr">
@@ -20401,7 +20401,7 @@
       </c>
       <c r="P180" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q180" t="n">
@@ -20501,7 +20501,7 @@
       </c>
       <c r="N181" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O181" t="inlineStr">
@@ -20511,7 +20511,7 @@
       </c>
       <c r="P181" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q181" t="n">
@@ -20611,7 +20611,7 @@
       </c>
       <c r="N182" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O182" t="inlineStr">
@@ -20621,7 +20621,7 @@
       </c>
       <c r="P182" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q182" t="n">
@@ -20721,7 +20721,7 @@
       </c>
       <c r="N183" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O183" t="inlineStr">
@@ -20731,7 +20731,7 @@
       </c>
       <c r="P183" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q183" t="n">
@@ -20831,7 +20831,7 @@
       </c>
       <c r="N184" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O184" t="inlineStr">
@@ -20841,7 +20841,7 @@
       </c>
       <c r="P184" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q184" t="n">
@@ -20941,7 +20941,7 @@
       </c>
       <c r="N185" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O185" t="inlineStr">
@@ -20951,7 +20951,7 @@
       </c>
       <c r="P185" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q185" t="n">
@@ -21051,7 +21051,7 @@
       </c>
       <c r="N186" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O186" t="inlineStr">
@@ -21061,7 +21061,7 @@
       </c>
       <c r="P186" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q186" t="n">
@@ -21161,7 +21161,7 @@
       </c>
       <c r="N187" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O187" t="inlineStr">
@@ -21171,7 +21171,7 @@
       </c>
       <c r="P187" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q187" t="n">
@@ -21271,7 +21271,7 @@
       </c>
       <c r="N188" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O188" t="inlineStr">
@@ -21281,7 +21281,7 @@
       </c>
       <c r="P188" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q188" t="n">
@@ -21381,7 +21381,7 @@
       </c>
       <c r="N189" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O189" t="inlineStr">
@@ -21391,7 +21391,7 @@
       </c>
       <c r="P189" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q189" t="n">
@@ -21491,7 +21491,7 @@
       </c>
       <c r="N190" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O190" t="inlineStr">
@@ -21501,7 +21501,7 @@
       </c>
       <c r="P190" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q190" t="n">
@@ -21601,7 +21601,7 @@
       </c>
       <c r="N191" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O191" t="inlineStr">
@@ -21611,7 +21611,7 @@
       </c>
       <c r="P191" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q191" t="n">
@@ -21711,7 +21711,7 @@
       </c>
       <c r="N192" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O192" t="inlineStr">
@@ -21721,7 +21721,7 @@
       </c>
       <c r="P192" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q192" t="n">
@@ -21821,7 +21821,7 @@
       </c>
       <c r="N193" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O193" t="inlineStr">
@@ -21831,7 +21831,7 @@
       </c>
       <c r="P193" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q193" t="n">
@@ -21931,7 +21931,7 @@
       </c>
       <c r="N194" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O194" t="inlineStr">
@@ -21941,7 +21941,7 @@
       </c>
       <c r="P194" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q194" t="n">
@@ -22041,7 +22041,7 @@
       </c>
       <c r="N195" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O195" t="inlineStr">
@@ -22051,7 +22051,7 @@
       </c>
       <c r="P195" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q195" t="n">
@@ -22151,7 +22151,7 @@
       </c>
       <c r="N196" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O196" t="inlineStr">
@@ -22161,7 +22161,7 @@
       </c>
       <c r="P196" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q196" t="n">
@@ -22261,7 +22261,7 @@
       </c>
       <c r="N197" t="inlineStr">
         <is>
-          <t>D5-LOCAL-20260726T101447Z</t>
+          <t>D5-LOCAL-20260727T034533Z</t>
         </is>
       </c>
       <c r="O197" t="inlineStr">
@@ -22271,7 +22271,7 @@
       </c>
       <c r="P197" t="inlineStr">
         <is>
-          <t>00d1d8f3e63aa9a40fa4c8bc85d532d175a6f2761b3fa7d04b06814d1ca96493</t>
+          <t>7b1ba852f0405944538e558e8df7fe74468789604eb0d90372b1762be3ca036a</t>
         </is>
       </c>
       <c r="Q197" t="n">

</xml_diff>